<commit_message>
fin task with pandas
</commit_message>
<xml_diff>
--- a/commissionByType.xlsx
+++ b/commissionByType.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,6 +427,16 @@
           <t>Объем транзакции</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Валюта</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Сумма в USD</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -437,6 +447,14 @@
       <c r="B2" t="n">
         <v>-1351.15</v>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>-19.24</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -446,6 +464,14 @@
       </c>
       <c r="B3" t="n">
         <v>-34586.09</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>-492.47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>